<commit_message>
v2: 12-month option for review and plan; planning view stays at 6 months
Seasonal naive now repeats last year beyond 12 months, so the previous
plan has no zero months.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuRRj27WbPXrKU9vXQExqg
</commit_message>
<xml_diff>
--- a/v2/demand-planning-sample-data.xlsx
+++ b/v2/demand-planning-sample-data.xlsx
@@ -57741,7 +57741,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -58437,7 +58437,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>295</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
@@ -59133,7 +59133,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
@@ -60177,7 +60177,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0</v>
+        <v>1042</v>
       </c>
       <c r="E97" t="n">
         <v>0</v>
@@ -60525,7 +60525,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0</v>
+        <v>919</v>
       </c>
       <c r="E109" t="n">
         <v>0</v>
@@ -65745,7 +65745,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E289" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v2: sample data with Presidents' Day and Memorial Day promotions
Promo months now show visible spikes above the statistical forecast.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuRRj27WbPXrKU9vXQExqg
</commit_message>
<xml_diff>
--- a/v2/demand-planning-sample-data.xlsx
+++ b/v2/demand-planning-sample-data.xlsx
@@ -1485,11 +1485,11 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>185</v>
+        <v>249</v>
       </c>
     </row>
     <row r="31">
@@ -1590,11 +1590,11 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>240</v>
+        <v>324</v>
       </c>
     </row>
     <row r="34">
@@ -2745,11 +2745,11 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G66" t="n">
-        <v>172</v>
+        <v>232</v>
       </c>
     </row>
     <row r="67">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G69" t="n">
-        <v>221</v>
+        <v>298</v>
       </c>
     </row>
     <row r="70">
@@ -4005,11 +4005,11 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G102" t="n">
-        <v>228</v>
+        <v>308</v>
       </c>
     </row>
     <row r="103">
@@ -4110,11 +4110,11 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G105" t="n">
-        <v>273</v>
+        <v>369</v>
       </c>
     </row>
     <row r="106">
@@ -9150,11 +9150,11 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G249" t="n">
-        <v>195</v>
+        <v>253</v>
       </c>
     </row>
     <row r="250">
@@ -10410,11 +10410,11 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G285" t="n">
-        <v>159</v>
+        <v>207</v>
       </c>
     </row>
     <row r="286">
@@ -11670,11 +11670,11 @@
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G321" t="n">
-        <v>240</v>
+        <v>312</v>
       </c>
     </row>
     <row r="322">
@@ -21124,7 +21124,7 @@
         </is>
       </c>
       <c r="G591" t="n">
-        <v>493</v>
+        <v>565</v>
       </c>
     </row>
     <row r="592">
@@ -22384,7 +22384,7 @@
         </is>
       </c>
       <c r="G627" t="n">
-        <v>401</v>
+        <v>460</v>
       </c>
     </row>
     <row r="628">
@@ -23644,7 +23644,7 @@
         </is>
       </c>
       <c r="G663" t="n">
-        <v>555</v>
+        <v>637</v>
       </c>
     </row>
     <row r="664">
@@ -24795,11 +24795,11 @@
       </c>
       <c r="F696" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G696" t="n">
-        <v>330</v>
+        <v>446</v>
       </c>
     </row>
     <row r="697">
@@ -24900,11 +24900,11 @@
       </c>
       <c r="F699" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G699" t="n">
-        <v>440</v>
+        <v>593</v>
       </c>
     </row>
     <row r="700">
@@ -26055,11 +26055,11 @@
       </c>
       <c r="F732" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G732" t="n">
-        <v>279</v>
+        <v>376</v>
       </c>
     </row>
     <row r="733">
@@ -26160,11 +26160,11 @@
       </c>
       <c r="F735" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G735" t="n">
-        <v>347</v>
+        <v>468</v>
       </c>
     </row>
     <row r="736">
@@ -27315,11 +27315,11 @@
       </c>
       <c r="F768" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G768" t="n">
-        <v>323</v>
+        <v>436</v>
       </c>
     </row>
     <row r="769">
@@ -27420,11 +27420,11 @@
       </c>
       <c r="F771" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G771" t="n">
-        <v>445</v>
+        <v>601</v>
       </c>
     </row>
     <row r="772">
@@ -32355,11 +32355,11 @@
       </c>
       <c r="F912" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G912" t="n">
-        <v>176</v>
+        <v>229</v>
       </c>
     </row>
     <row r="913">
@@ -32460,11 +32460,11 @@
       </c>
       <c r="F915" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G915" t="n">
-        <v>251</v>
+        <v>327</v>
       </c>
     </row>
     <row r="916">
@@ -33615,11 +33615,11 @@
       </c>
       <c r="F948" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G948" t="n">
-        <v>147</v>
+        <v>192</v>
       </c>
     </row>
     <row r="949">
@@ -33720,11 +33720,11 @@
       </c>
       <c r="F951" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G951" t="n">
-        <v>202</v>
+        <v>263</v>
       </c>
     </row>
     <row r="952">
@@ -34875,11 +34875,11 @@
       </c>
       <c r="F984" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G984" t="n">
-        <v>216</v>
+        <v>281</v>
       </c>
     </row>
     <row r="985">
@@ -34980,11 +34980,11 @@
       </c>
       <c r="F987" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G987" t="n">
-        <v>282</v>
+        <v>366</v>
       </c>
     </row>
     <row r="988">
@@ -46538,7 +46538,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="E2" t="n">
         <v>70</v>
@@ -46564,7 +46564,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>281</v>
+        <v>325</v>
       </c>
       <c r="E3" t="n">
         <v>60</v>
@@ -46590,7 +46590,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>446</v>
+        <v>485</v>
       </c>
       <c r="E4" t="n">
         <v>80</v>
@@ -46694,7 +46694,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>342</v>
+        <v>371</v>
       </c>
       <c r="E8" t="n">
         <v>50</v>
@@ -46720,7 +46720,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>306</v>
+        <v>336</v>
       </c>
       <c r="E9" t="n">
         <v>40</v>
@@ -46746,7 +46746,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>421</v>
+        <v>474</v>
       </c>
       <c r="E10" t="n">
         <v>60</v>
@@ -47006,7 +47006,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>453</v>
+        <v>478</v>
       </c>
       <c r="E20" t="n">
         <v>110</v>
@@ -47032,7 +47032,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="E21" t="n">
         <v>90</v>
@@ -47058,7 +47058,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>444</v>
+        <v>470</v>
       </c>
       <c r="E22" t="n">
         <v>130</v>
@@ -47084,7 +47084,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>307</v>
+        <v>365</v>
       </c>
       <c r="E23" t="n">
         <v>110</v>
@@ -47110,7 +47110,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>301</v>
+        <v>357</v>
       </c>
       <c r="E24" t="n">
         <v>90</v>
@@ -47136,7 +47136,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>389</v>
+        <v>418</v>
       </c>
       <c r="E25" t="n">
         <v>130</v>
@@ -47240,7 +47240,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>321</v>
+        <v>345</v>
       </c>
       <c r="E29" t="n">
         <v>70</v>
@@ -47266,7 +47266,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="E30" t="n">
         <v>50</v>
@@ -47292,7 +47292,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>386</v>
+        <v>423</v>
       </c>
       <c r="E31" t="n">
         <v>80</v>
@@ -47775,7 +47775,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1750</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="3">
@@ -47790,7 +47790,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1960</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="4">
@@ -47805,7 +47805,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1610</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="5">
@@ -47820,7 +47820,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1540</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="6">
@@ -47835,7 +47835,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1560</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="7">
@@ -47850,7 +47850,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1700</v>
+        <v>1730</v>
       </c>
     </row>
     <row r="8">
@@ -47865,7 +47865,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1800</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="9">
@@ -47880,7 +47880,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2150</v>
+        <v>2670</v>
       </c>
     </row>
     <row r="10">
@@ -47895,7 +47895,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1900</v>
+        <v>1940</v>
       </c>
     </row>
     <row r="11">
@@ -47910,7 +47910,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1970</v>
+        <v>2010</v>
       </c>
     </row>
     <row r="12">
@@ -47925,7 +47925,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1990</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="13">
@@ -47940,7 +47940,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2230</v>
+        <v>2270</v>
       </c>
     </row>
     <row r="14">
@@ -48015,7 +48015,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3080</v>
+        <v>3580</v>
       </c>
     </row>
     <row r="19">
@@ -48060,7 +48060,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4370</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="22">
@@ -48442,7 +48442,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>173</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7">
@@ -48502,7 +48502,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>231</v>
+        <v>315</v>
       </c>
     </row>
     <row r="10">
@@ -48682,7 +48682,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>175</v>
+        <v>233</v>
       </c>
     </row>
     <row r="19">
@@ -48742,7 +48742,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>203</v>
+        <v>282</v>
       </c>
     </row>
     <row r="22">
@@ -48922,7 +48922,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
     </row>
     <row r="31">
@@ -48982,7 +48982,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>284</v>
+        <v>375</v>
       </c>
     </row>
     <row r="34">
@@ -49942,7 +49942,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>218</v>
+        <v>272</v>
       </c>
     </row>
     <row r="82">
@@ -50182,7 +50182,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>167</v>
+        <v>213</v>
       </c>
     </row>
     <row r="94">
@@ -50422,7 +50422,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>228</v>
+        <v>299</v>
       </c>
     </row>
     <row r="106">
@@ -52462,7 +52462,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>485</v>
+        <v>555</v>
       </c>
     </row>
     <row r="208">
@@ -52702,7 +52702,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>382</v>
+        <v>438</v>
       </c>
     </row>
     <row r="220">
@@ -52942,7 +52942,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>572</v>
+        <v>656</v>
       </c>
     </row>
     <row r="232">
@@ -53122,7 +53122,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>327</v>
+        <v>440</v>
       </c>
     </row>
     <row r="241">
@@ -53182,7 +53182,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>484</v>
+        <v>630</v>
       </c>
     </row>
     <row r="244">
@@ -53362,7 +53362,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>284</v>
+        <v>378</v>
       </c>
     </row>
     <row r="253">
@@ -53422,7 +53422,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>344</v>
+        <v>462</v>
       </c>
     </row>
     <row r="256">
@@ -53602,7 +53602,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>301</v>
+        <v>412</v>
       </c>
     </row>
     <row r="265">
@@ -53662,7 +53662,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>437</v>
+        <v>590</v>
       </c>
     </row>
     <row r="268">
@@ -54562,7 +54562,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>175</v>
+        <v>227</v>
       </c>
     </row>
     <row r="313">
@@ -54622,7 +54622,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>244</v>
+        <v>319</v>
       </c>
     </row>
     <row r="316">
@@ -54802,7 +54802,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>136</v>
+        <v>180</v>
       </c>
     </row>
     <row r="325">
@@ -54862,7 +54862,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>218</v>
+        <v>276</v>
       </c>
     </row>
     <row r="328">
@@ -55042,7 +55042,7 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>236</v>
+        <v>297</v>
       </c>
     </row>
     <row r="337">
@@ -55102,7 +55102,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>288</v>
+        <v>368</v>
       </c>
     </row>
     <row r="340">
@@ -60902,7 +60902,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>413</v>
+        <v>406</v>
       </c>
       <c r="E122" t="n">
         <v>0</v>
@@ -60931,7 +60931,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>536</v>
+        <v>494</v>
       </c>
       <c r="E123" t="n">
         <v>0</v>
@@ -60960,7 +60960,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>383</v>
+        <v>414</v>
       </c>
       <c r="E124" t="n">
         <v>0</v>
@@ -60989,7 +60989,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="E125" t="n">
         <v>0</v>
@@ -61018,7 +61018,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>376</v>
+        <v>408</v>
       </c>
       <c r="E126" t="n">
         <v>0</v>
@@ -61047,7 +61047,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>422</v>
+        <v>413</v>
       </c>
       <c r="E127" t="n">
         <v>0</v>
@@ -61076,7 +61076,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>416</v>
+        <v>446</v>
       </c>
       <c r="E128" t="n">
         <v>0</v>
@@ -61105,7 +61105,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="E129" t="n">
         <v>0</v>
@@ -61134,7 +61134,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E130" t="n">
         <v>0</v>
@@ -61163,7 +61163,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>438</v>
+        <v>462</v>
       </c>
       <c r="E131" t="n">
         <v>0</v>
@@ -61221,7 +61221,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>483</v>
+        <v>493</v>
       </c>
       <c r="E133" t="n">
         <v>0</v>
@@ -61250,7 +61250,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>361</v>
+        <v>383</v>
       </c>
       <c r="E134" t="n">
         <v>0</v>
@@ -61279,7 +61279,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>432</v>
+        <v>458</v>
       </c>
       <c r="E135" t="n">
         <v>0</v>
@@ -61308,7 +61308,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>347</v>
+        <v>368</v>
       </c>
       <c r="E136" t="n">
         <v>0</v>
@@ -61337,7 +61337,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>348</v>
+        <v>370</v>
       </c>
       <c r="E137" t="n">
         <v>0</v>
@@ -61366,7 +61366,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>340</v>
+        <v>367</v>
       </c>
       <c r="E138" t="n">
         <v>0</v>
@@ -61395,7 +61395,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>373</v>
+        <v>396</v>
       </c>
       <c r="E139" t="n">
         <v>0</v>
@@ -61424,7 +61424,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>381</v>
+        <v>405</v>
       </c>
       <c r="E140" t="n">
         <v>0</v>
@@ -61453,7 +61453,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>415</v>
+        <v>448</v>
       </c>
       <c r="E141" t="n">
         <v>0</v>
@@ -61482,7 +61482,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>383</v>
+        <v>408</v>
       </c>
       <c r="E142" t="n">
         <v>0</v>
@@ -61511,7 +61511,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>401</v>
+        <v>427</v>
       </c>
       <c r="E143" t="n">
         <v>0</v>
@@ -61540,7 +61540,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>364</v>
+        <v>389</v>
       </c>
       <c r="E144" t="n">
         <v>0</v>
@@ -61569,7 +61569,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>430</v>
+        <v>461</v>
       </c>
       <c r="E145" t="n">
         <v>0</v>
@@ -61598,7 +61598,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="E146" t="n">
         <v>0</v>
@@ -61627,7 +61627,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="E147" t="n">
         <v>0</v>
@@ -61656,7 +61656,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E148" t="n">
         <v>0</v>
@@ -61685,7 +61685,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E149" t="n">
         <v>0</v>
@@ -61714,7 +61714,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E150" t="n">
         <v>0</v>
@@ -61743,7 +61743,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E151" t="n">
         <v>0</v>
@@ -61772,7 +61772,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="E152" t="n">
         <v>0</v>
@@ -61801,7 +61801,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="E153" t="n">
         <v>0</v>
@@ -61830,7 +61830,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="E154" t="n">
         <v>0</v>
@@ -61859,7 +61859,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="E155" t="n">
         <v>0</v>
@@ -61888,7 +61888,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="E156" t="n">
         <v>0</v>
@@ -61917,7 +61917,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="E157" t="n">
         <v>0</v>
@@ -61946,7 +61946,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>438</v>
+        <v>455</v>
       </c>
       <c r="E158" t="n">
         <v>0</v>
@@ -61975,7 +61975,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>667</v>
+        <v>694</v>
       </c>
       <c r="E159" t="n">
         <v>0</v>
@@ -62004,7 +62004,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>397</v>
+        <v>413</v>
       </c>
       <c r="E160" t="n">
         <v>0</v>
@@ -62033,7 +62033,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>447</v>
+        <v>466</v>
       </c>
       <c r="E161" t="n">
         <v>0</v>
@@ -62062,7 +62062,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>396</v>
+        <v>413</v>
       </c>
       <c r="E162" t="n">
         <v>0</v>
@@ -62091,7 +62091,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="E163" t="n">
         <v>0</v>
@@ -62120,7 +62120,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>407</v>
+        <v>424</v>
       </c>
       <c r="E164" t="n">
         <v>0</v>
@@ -62149,7 +62149,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>580</v>
+        <v>607</v>
       </c>
       <c r="E165" t="n">
         <v>0</v>
@@ -62178,7 +62178,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>403</v>
+        <v>419</v>
       </c>
       <c r="E166" t="n">
         <v>0</v>
@@ -62207,7 +62207,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>431</v>
+        <v>449</v>
       </c>
       <c r="E167" t="n">
         <v>0</v>
@@ -62236,7 +62236,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>424</v>
+        <v>443</v>
       </c>
       <c r="E168" t="n">
         <v>0</v>
@@ -62265,7 +62265,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>440</v>
+        <v>461</v>
       </c>
       <c r="E169" t="n">
         <v>0</v>
@@ -62294,7 +62294,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="E170" t="n">
         <v>0</v>
@@ -62323,7 +62323,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>533</v>
+        <v>542</v>
       </c>
       <c r="E171" t="n">
         <v>0</v>
@@ -62352,7 +62352,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="E172" t="n">
         <v>0</v>
@@ -62381,7 +62381,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="E173" t="n">
         <v>0</v>
@@ -62410,7 +62410,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="E174" t="n">
         <v>0</v>
@@ -62439,7 +62439,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="E175" t="n">
         <v>0</v>
@@ -62468,7 +62468,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="E176" t="n">
         <v>0</v>
@@ -62497,7 +62497,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>434</v>
+        <v>445</v>
       </c>
       <c r="E177" t="n">
         <v>0</v>
@@ -62526,7 +62526,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="E178" t="n">
         <v>0</v>
@@ -62555,7 +62555,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="E179" t="n">
         <v>0</v>
@@ -62584,7 +62584,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="E180" t="n">
         <v>0</v>
@@ -62613,7 +62613,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="E181" t="n">
         <v>0</v>
@@ -63686,7 +63686,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="E218" t="n">
         <v>0</v>
@@ -63715,7 +63715,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="E219" t="n">
         <v>0</v>
@@ -63744,7 +63744,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E220" t="n">
         <v>0</v>
@@ -63773,7 +63773,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E221" t="n">
         <v>0</v>
@@ -63802,7 +63802,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>148</v>
+        <v>192</v>
       </c>
       <c r="E222" t="n">
         <v>0</v>
@@ -63831,7 +63831,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="E223" t="n">
         <v>0</v>
@@ -63889,7 +63889,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>191</v>
+        <v>263</v>
       </c>
       <c r="E225" t="n">
         <v>0</v>
@@ -63918,7 +63918,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E226" t="n">
         <v>0</v>
@@ -63947,7 +63947,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>197</v>
+        <v>178</v>
       </c>
       <c r="E227" t="n">
         <v>0</v>
@@ -63976,7 +63976,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="E228" t="n">
         <v>0</v>
@@ -64034,7 +64034,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="E230" t="n">
         <v>0</v>
@@ -64063,7 +64063,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="E231" t="n">
         <v>0</v>
@@ -64092,7 +64092,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="E232" t="n">
         <v>0</v>
@@ -64121,7 +64121,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>225</v>
+        <v>251</v>
       </c>
       <c r="E233" t="n">
         <v>0</v>
@@ -64150,7 +64150,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>207</v>
+        <v>281</v>
       </c>
       <c r="E234" t="n">
         <v>0</v>
@@ -64179,7 +64179,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E235" t="n">
         <v>0</v>
@@ -64208,7 +64208,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>247</v>
+        <v>229</v>
       </c>
       <c r="E236" t="n">
         <v>0</v>
@@ -64237,7 +64237,7 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>279</v>
+        <v>366</v>
       </c>
       <c r="E237" t="n">
         <v>0</v>
@@ -64266,7 +64266,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>237</v>
+        <v>261</v>
       </c>
       <c r="E238" t="n">
         <v>0</v>
@@ -64295,7 +64295,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E239" t="n">
         <v>0</v>
@@ -64324,7 +64324,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="E240" t="n">
         <v>0</v>
@@ -64353,7 +64353,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="E241" t="n">
         <v>0</v>
@@ -64382,7 +64382,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="E242" t="n">
         <v>0</v>
@@ -64411,7 +64411,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="E243" t="n">
         <v>0</v>
@@ -64440,7 +64440,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="E244" t="n">
         <v>0</v>
@@ -64469,7 +64469,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="E245" t="n">
         <v>0</v>
@@ -64498,7 +64498,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="E246" t="n">
         <v>0</v>
@@ -64527,7 +64527,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="E247" t="n">
         <v>0</v>
@@ -64556,7 +64556,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="E248" t="n">
         <v>0</v>
@@ -64585,7 +64585,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>270</v>
+        <v>287</v>
       </c>
       <c r="E249" t="n">
         <v>0</v>
@@ -64614,7 +64614,7 @@
         </is>
       </c>
       <c r="D250" t="n">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="E250" t="n">
         <v>0</v>
@@ -64643,7 +64643,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="E251" t="n">
         <v>0</v>
@@ -64672,7 +64672,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="E252" t="n">
         <v>0</v>
@@ -64701,7 +64701,7 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>311</v>
+        <v>327</v>
       </c>
       <c r="E253" t="n">
         <v>0</v>
@@ -66818,7 +66818,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="E326" t="n">
         <v>0</v>
@@ -66847,7 +66847,7 @@
         </is>
       </c>
       <c r="D327" t="n">
-        <v>207</v>
+        <v>229</v>
       </c>
       <c r="E327" t="n">
         <v>0</v>
@@ -66856,7 +66856,7 @@
         <v>0</v>
       </c>
       <c r="G327" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="328">
@@ -66876,7 +66876,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="E328" t="n">
         <v>0</v>
@@ -66905,7 +66905,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>156</v>
+        <v>187</v>
       </c>
       <c r="E329" t="n">
         <v>0</v>
@@ -66934,7 +66934,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>153</v>
+        <v>197</v>
       </c>
       <c r="E330" t="n">
         <v>0</v>
@@ -66963,7 +66963,7 @@
         </is>
       </c>
       <c r="D331" t="n">
-        <v>176</v>
+        <v>196</v>
       </c>
       <c r="E331" t="n">
         <v>0</v>
@@ -66992,7 +66992,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>172</v>
+        <v>206</v>
       </c>
       <c r="E332" t="n">
         <v>0</v>
@@ -67021,7 +67021,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>198</v>
+        <v>256</v>
       </c>
       <c r="E333" t="n">
         <v>0</v>
@@ -67050,7 +67050,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>182</v>
+        <v>226</v>
       </c>
       <c r="E334" t="n">
         <v>0</v>
@@ -67079,7 +67079,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>185</v>
+        <v>215</v>
       </c>
       <c r="E335" t="n">
         <v>0</v>
@@ -67108,7 +67108,7 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>178</v>
+        <v>227</v>
       </c>
       <c r="E336" t="n">
         <v>0</v>
@@ -67137,7 +67137,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>197</v>
+        <v>257</v>
       </c>
       <c r="E337" t="n">
         <v>0</v>
@@ -69979,7 +69979,7 @@
         </is>
       </c>
       <c r="D435" t="n">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="E435" t="n">
         <v>0</v>
@@ -70008,7 +70008,7 @@
         </is>
       </c>
       <c r="D436" t="n">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="E436" t="n">
         <v>0</v>
@@ -70037,7 +70037,7 @@
         </is>
       </c>
       <c r="D437" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E437" t="n">
         <v>0</v>
@@ -70066,7 +70066,7 @@
         </is>
       </c>
       <c r="D438" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E438" t="n">
         <v>0</v>
@@ -70095,7 +70095,7 @@
         </is>
       </c>
       <c r="D439" t="n">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E439" t="n">
         <v>0</v>
@@ -70124,7 +70124,7 @@
         </is>
       </c>
       <c r="D440" t="n">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E440" t="n">
         <v>0</v>
@@ -70153,7 +70153,7 @@
         </is>
       </c>
       <c r="D441" t="n">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="E441" t="n">
         <v>0</v>
@@ -70182,7 +70182,7 @@
         </is>
       </c>
       <c r="D442" t="n">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E442" t="n">
         <v>0</v>
@@ -70211,7 +70211,7 @@
         </is>
       </c>
       <c r="D443" t="n">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="E443" t="n">
         <v>0</v>
@@ -70240,7 +70240,7 @@
         </is>
       </c>
       <c r="D444" t="n">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="E444" t="n">
         <v>0</v>
@@ -70269,7 +70269,7 @@
         </is>
       </c>
       <c r="D445" t="n">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E445" t="n">
         <v>0</v>
@@ -70298,7 +70298,7 @@
         </is>
       </c>
       <c r="D446" t="n">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="E446" t="n">
         <v>0</v>
@@ -70327,7 +70327,7 @@
         </is>
       </c>
       <c r="D447" t="n">
-        <v>225</v>
+        <v>203</v>
       </c>
       <c r="E447" t="n">
         <v>0</v>
@@ -70356,7 +70356,7 @@
         </is>
       </c>
       <c r="D448" t="n">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="E448" t="n">
         <v>0</v>
@@ -70385,7 +70385,7 @@
         </is>
       </c>
       <c r="D449" t="n">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="E449" t="n">
         <v>0</v>
@@ -70414,7 +70414,7 @@
         </is>
       </c>
       <c r="D450" t="n">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="E450" t="n">
         <v>0</v>
@@ -70443,7 +70443,7 @@
         </is>
       </c>
       <c r="D451" t="n">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="E451" t="n">
         <v>0</v>
@@ -70472,7 +70472,7 @@
         </is>
       </c>
       <c r="D452" t="n">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="E452" t="n">
         <v>0</v>
@@ -70501,7 +70501,7 @@
         </is>
       </c>
       <c r="D453" t="n">
-        <v>216</v>
+        <v>312</v>
       </c>
       <c r="E453" t="n">
         <v>0</v>
@@ -70530,7 +70530,7 @@
         </is>
       </c>
       <c r="D454" t="n">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="E454" t="n">
         <v>0</v>
@@ -70559,7 +70559,7 @@
         </is>
       </c>
       <c r="D455" t="n">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="E455" t="n">
         <v>0</v>
@@ -70588,7 +70588,7 @@
         </is>
       </c>
       <c r="D456" t="n">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="E456" t="n">
         <v>0</v>
@@ -70617,7 +70617,7 @@
         </is>
       </c>
       <c r="D457" t="n">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="E457" t="n">
         <v>0</v>
@@ -70646,7 +70646,7 @@
         </is>
       </c>
       <c r="D458" t="n">
-        <v>161</v>
+        <v>181</v>
       </c>
       <c r="E458" t="n">
         <v>0</v>
@@ -70675,7 +70675,7 @@
         </is>
       </c>
       <c r="D459" t="n">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="E459" t="n">
         <v>0</v>
@@ -70704,7 +70704,7 @@
         </is>
       </c>
       <c r="D460" t="n">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="E460" t="n">
         <v>0</v>
@@ -70733,7 +70733,7 @@
         </is>
       </c>
       <c r="D461" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E461" t="n">
         <v>0</v>
@@ -70762,7 +70762,7 @@
         </is>
       </c>
       <c r="D462" t="n">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E462" t="n">
         <v>0</v>
@@ -70791,7 +70791,7 @@
         </is>
       </c>
       <c r="D463" t="n">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E463" t="n">
         <v>0</v>
@@ -70849,7 +70849,7 @@
         </is>
       </c>
       <c r="D465" t="n">
-        <v>187</v>
+        <v>253</v>
       </c>
       <c r="E465" t="n">
         <v>0</v>
@@ -70878,7 +70878,7 @@
         </is>
       </c>
       <c r="D466" t="n">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="E466" t="n">
         <v>0</v>
@@ -70907,7 +70907,7 @@
         </is>
       </c>
       <c r="D467" t="n">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E467" t="n">
         <v>0</v>
@@ -70936,7 +70936,7 @@
         </is>
       </c>
       <c r="D468" t="n">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="E468" t="n">
         <v>0</v>
@@ -70965,7 +70965,7 @@
         </is>
       </c>
       <c r="D469" t="n">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E469" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v2: sample consensus input more accurate in Jul-Sep 2026 (positive FVA)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuRRj27WbPXrKU9vXQExqg
</commit_message>
<xml_diff>
--- a/v2/demand-planning-sample-data.xlsx
+++ b/v2/demand-planning-sample-data.xlsx
@@ -55382,7 +55382,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>358</v>
+        <v>329</v>
       </c>
     </row>
     <row r="354">
@@ -55402,7 +55402,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>354</v>
+        <v>318</v>
       </c>
     </row>
     <row r="355">
@@ -55422,7 +55422,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>289</v>
+        <v>283</v>
       </c>
     </row>
     <row r="356">
@@ -55622,7 +55622,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>249</v>
+        <v>241</v>
       </c>
     </row>
     <row r="366">
@@ -55642,7 +55642,7 @@
         </is>
       </c>
       <c r="D366" t="n">
-        <v>270</v>
+        <v>254</v>
       </c>
     </row>
     <row r="367">
@@ -55662,7 +55662,7 @@
         </is>
       </c>
       <c r="D367" t="n">
-        <v>293</v>
+        <v>276</v>
       </c>
     </row>
     <row r="368">
@@ -55862,7 +55862,7 @@
         </is>
       </c>
       <c r="D377" t="n">
-        <v>377</v>
+        <v>360</v>
       </c>
     </row>
     <row r="378">
@@ -55882,7 +55882,7 @@
         </is>
       </c>
       <c r="D378" t="n">
-        <v>362</v>
+        <v>335</v>
       </c>
     </row>
     <row r="379">
@@ -55902,7 +55902,7 @@
         </is>
       </c>
       <c r="D379" t="n">
-        <v>323</v>
+        <v>331</v>
       </c>
     </row>
     <row r="380">
@@ -56102,7 +56102,7 @@
         </is>
       </c>
       <c r="D389" t="n">
-        <v>205</v>
+        <v>187</v>
       </c>
     </row>
     <row r="390">
@@ -56122,7 +56122,7 @@
         </is>
       </c>
       <c r="D390" t="n">
-        <v>210</v>
+        <v>197</v>
       </c>
     </row>
     <row r="391">
@@ -56142,7 +56142,7 @@
         </is>
       </c>
       <c r="D391" t="n">
-        <v>203</v>
+        <v>181</v>
       </c>
     </row>
     <row r="392">
@@ -56342,7 +56342,7 @@
         </is>
       </c>
       <c r="D401" t="n">
-        <v>150</v>
+        <v>141</v>
       </c>
     </row>
     <row r="402">
@@ -56362,7 +56362,7 @@
         </is>
       </c>
       <c r="D402" t="n">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="403">
@@ -56382,7 +56382,7 @@
         </is>
       </c>
       <c r="D403" t="n">
-        <v>133</v>
+        <v>148</v>
       </c>
     </row>
     <row r="404">
@@ -56582,7 +56582,7 @@
         </is>
       </c>
       <c r="D413" t="n">
-        <v>230</v>
+        <v>211</v>
       </c>
     </row>
     <row r="414">
@@ -56602,7 +56602,7 @@
         </is>
       </c>
       <c r="D414" t="n">
-        <v>227</v>
+        <v>210</v>
       </c>
     </row>
     <row r="415">
@@ -56622,7 +56622,7 @@
         </is>
       </c>
       <c r="D415" t="n">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="416">
@@ -56822,7 +56822,7 @@
         </is>
       </c>
       <c r="D425" t="n">
-        <v>1182</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="426">
@@ -56842,7 +56842,7 @@
         </is>
       </c>
       <c r="D426" t="n">
-        <v>1027</v>
+        <v>951</v>
       </c>
     </row>
     <row r="427">
@@ -56862,7 +56862,7 @@
         </is>
       </c>
       <c r="D427" t="n">
-        <v>1063</v>
+        <v>984</v>
       </c>
     </row>
     <row r="428">
@@ -57062,7 +57062,7 @@
         </is>
       </c>
       <c r="D437" t="n">
-        <v>868</v>
+        <v>844</v>
       </c>
     </row>
     <row r="438">
@@ -57082,7 +57082,7 @@
         </is>
       </c>
       <c r="D438" t="n">
-        <v>727</v>
+        <v>749</v>
       </c>
     </row>
     <row r="439">
@@ -57102,7 +57102,7 @@
         </is>
       </c>
       <c r="D439" t="n">
-        <v>763</v>
+        <v>783</v>
       </c>
     </row>
     <row r="440">
@@ -57302,7 +57302,7 @@
         </is>
       </c>
       <c r="D449" t="n">
-        <v>1111</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="450">
@@ -57322,7 +57322,7 @@
         </is>
       </c>
       <c r="D450" t="n">
-        <v>1411</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="451">
@@ -57342,7 +57342,7 @@
         </is>
       </c>
       <c r="D451" t="n">
-        <v>1073</v>
+        <v>1088</v>
       </c>
     </row>
   </sheetData>

</xml_diff>